<commit_message>
Sjekkpakker: nytt format etter testing
- Format fra testen av sjekkpakker: kantlinjer, sammenslåtte celler,
  omskrevne instrukser
- «Om kilden» erstattet av «Avvik / betalingsmur / uventet»
- Ny kolonne «Hvor i kilden»: side, §, artikkel, avsnitt eller
  overskrift kreves for verifisert og delvis
- Regler og veiledning oppdatert tilsvarende
- Merknad om offentlig navn på «Sjekket av»
</commit_message>
<xml_diff>
--- a/dugnad/sjekkpakker/DEM-01.xlsx
+++ b/dugnad/sjekkpakker/DEM-01.xlsx
@@ -20,7 +20,7 @@
     <comment ref="B4" authorId="0">
       <text>
         <r>
-          <t>Kallenavn eller GitHub-navn. Det kan bli stående offentlig i kilderegisteret.</t>
+          <t>Navnet du vil stå med offentlig: fullt navn, kallenavn eller GitHub-navn. Det blir stående i kilderegisteret på GitHub og kan ikke fjernes helt i ettertid.</t>
         </r>
       </text>
     </comment>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="212">
   <si>
     <t>Sjekkpakke DEM-01: Påvirkning og designet manipulasjon</t>
   </si>
@@ -64,7 +64,10 @@
     <t>3</t>
   </si>
   <si>
-    <t>Les det som er relevant, og sammenlign med «Rapporten sier». Sett «Status» og skriv kort i «Om kilden» hvordan du sjekket og hva som eventuelt avviker.</t>
+    <t>Les det som er relevant, og sammenlign med «Rapporten sier». Sett «Status», og skriv i «Avvik» hvis noe avviker, ligger bak betalingsmur eller er uventet.</t>
+  </si>
+  <si>
+    <t>Er status «verifisert» eller «delvis», skriv i «Hvor i kilden» hvor det står: side (rapport, bok, artikkel), § og ledd (lov), artikkel og nummer (EU-rett), avsnitt (dom) eller overskrift (nettside). Da kan neste person slå rett opp.</t>
   </si>
   <si>
     <t>4</t>
@@ -94,13 +97,13 @@
     <t>verifisert</t>
   </si>
   <si>
-    <t>Du har åpnet primærkilden, og den sier det påstanden bygger på.</t>
+    <t>Du har lest det relevante i primærkilden, og den sier det påstanden bygger på.</t>
   </si>
   <si>
     <t>delvis</t>
   </si>
   <si>
-    <t>Stemmer, men med avvik. Skriv avviket i «Om kilden».</t>
+    <t>Stemmer, men med avvik. Skriv avviket i «Avvik».</t>
   </si>
   <si>
     <t>sekundær</t>
@@ -157,13 +160,13 @@
     <t>A Aktualitet</t>
   </si>
   <si>
-    <t>Er det fortsatt gyldig? 0 utdatert (motbevist, erstattet, loven endret) eller ikke sjekket · 1 usikker gyldighet (feltet har endret seg mye siden, f.eks. studier av eldre KI-modeller) · 2 gyldig, ingen kjent nyere forskning sier noe annet, uansett alder · 3 fersk (gjelder dagens situasjon) eller bekreftet av nyere forskning. Bekreftelsen kan stå i kommentaren.</t>
+    <t>Er det fortsatt gyldig? 0 utdatert (motbevist, erstattet, lovendring) eller ikke sjekket · 1 usikker gyldighet (feltet har endret seg mye siden, f.eks. studier av eldre KI-modeller) · 2 gyldig, ingen kjent nyere forskning sier noe annet, uansett alder · 3 fersk (gjelder dagens situasjon) eller bekreftet av nyere forskning. Bekreftelsen kan stå i kommentaren.</t>
   </si>
   <si>
     <t>Husk</t>
   </si>
   <si>
-    <t>Aldri dikt opp. Tall, datoer og navn tas fra kilden, ikke fra hukommelsen.</t>
+    <t>Ha integritet.</t>
   </si>
   <si>
     <t>Skill mellom «viser», «tyder på» og «antyder», og mellom én studie og konsensus. En påstand kan ha riktig kilde og likevel si mer enn kilden gjør.</t>
@@ -205,13 +208,16 @@
     <t>Status ▾</t>
   </si>
   <si>
+    <t>Hvor i kilden (s., §, art., avsnitt)</t>
+  </si>
+  <si>
     <t>Riktig eller ny lenke / DOI</t>
   </si>
   <si>
     <t>Fagfelle-vurdert ▾</t>
   </si>
   <si>
-    <t>Om kilden: hvordan du sjekket, hva som avviker</t>
+    <t>Avvik / betalingsmur / uventet</t>
   </si>
   <si>
     <t>E ▾</t>
@@ -666,6 +672,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+  </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -698,12 +707,17 @@
       <color rgb="FF1F5FA8"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEEEEE"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -726,7 +740,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -734,36 +748,66 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="hair"/>
+      <right style="hair"/>
+      <top style="hair"/>
+      <bottom style="hair"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1105,256 +1149,291 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="90" customWidth="1"/>
+    <col min="2" max="2" width="91.45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="2"/>
+    </row>
+    <row r="2" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="4"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+    </row>
+    <row r="4" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="B4" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="B5" s="9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
+    </row>
+    <row r="7" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="B7" s="12" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="13" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="13" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="3" t="s">
+    </row>
+    <row r="12" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="B12" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="3" t="s">
+    </row>
+    <row r="13" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="B13" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="3" t="s">
+    </row>
+    <row r="14" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+    <row r="15" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+    </row>
+    <row r="17" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="12" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="B18" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="3" t="s">
+    </row>
+    <row r="19" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="B19" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="3" t="s">
+    </row>
+    <row r="20" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="B20" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="3" t="s">
+    </row>
+    <row r="21" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+      <c r="B21" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="3" t="s">
+    </row>
+    <row r="22" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="13" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
+    <row r="23" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="6" t="s">
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="10"/>
+      <c r="B24" s="10"/>
+    </row>
+    <row r="25" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+      <c r="B25" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="3" t="s">
+    </row>
+    <row r="26" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+      <c r="B26" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="B26" s="3" t="s">
+    </row>
+    <row r="27" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
+      <c r="B27" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B27" s="3" t="s">
+    </row>
+    <row r="28" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
+      <c r="B28" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="3" t="s">
+    </row>
+    <row r="29" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
+      <c r="B29" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="B29" s="3" t="s">
+    </row>
+    <row r="30" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
+      <c r="B30" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B31" s="6" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B32" s="3" t="s">
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="10"/>
+      <c r="B31" s="10"/>
+    </row>
+    <row r="32" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B33" s="3" t="s">
+      <c r="B32" s="12" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B33" s="13" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B34" s="3" t="s">
+    <row r="34" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B34" s="13" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="35" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B35" s="3" t="s">
+    <row r="35" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B35" s="13" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
+    <row r="36" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B36" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="B36" s="3" t="s">
+    </row>
+    <row r="37" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="7" t="s">
         <v>49</v>
       </c>
+      <c r="B37" s="13" t="s">
+        <v>50</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <legacyDrawing r:id="rId2"/>
@@ -1363,7 +1442,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1374,951 +1453,981 @@
     <col min="6" max="6" width="60" customWidth="1"/>
     <col min="7" max="7" width="36" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
-    <col min="10" max="10" width="11" customWidth="1"/>
-    <col min="11" max="11" width="36" customWidth="1"/>
-    <col min="12" max="16" width="5" customWidth="1"/>
-    <col min="17" max="17" width="40" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="26" customWidth="1"/>
+    <col min="11" max="11" width="11" customWidth="1"/>
+    <col min="12" max="12" width="36" customWidth="1"/>
+    <col min="13" max="17" width="5" customWidth="1"/>
+    <col min="18" max="18" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="7" t="s">
+    <row r="1" ht="32" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="B1" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="C1" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="D1" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="E1" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="F1" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="G1" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="H1" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="I1" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="J1" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="K1" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="L1" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="M1" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="N1" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="O1" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="P1" s="15" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+      <c r="Q1" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="R1" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="9" t="s">
+    </row>
+    <row r="2" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="B2" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="E2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5"/>
-    </row>
-    <row r="3" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="C2" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="D2" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="E2" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="17"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="17"/>
+    </row>
+    <row r="3" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="B3" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="C3" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="D3" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="E3" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-    </row>
-    <row r="4" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+      <c r="F3" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="G3" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
+      <c r="K3" s="17"/>
+      <c r="L3" s="17"/>
+      <c r="M3" s="17"/>
+      <c r="N3" s="17"/>
+      <c r="O3" s="17"/>
+      <c r="P3" s="17"/>
+      <c r="Q3" s="17"/>
+      <c r="R3" s="17"/>
+    </row>
+    <row r="4" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="B4" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="C4" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="F4" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="G4" s="9" t="s">
+      <c r="D4" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
-    </row>
-    <row r="5" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="E4" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="F4" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G4" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="17"/>
+      <c r="L4" s="17"/>
+      <c r="M4" s="17"/>
+      <c r="N4" s="17"/>
+      <c r="O4" s="17"/>
+      <c r="P4" s="17"/>
+      <c r="Q4" s="17"/>
+      <c r="R4" s="17"/>
+    </row>
+    <row r="5" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="B5" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="C5" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="D5" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="E5" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="5"/>
-    </row>
-    <row r="6" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+      <c r="F5" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="G5" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="C6" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-    </row>
-    <row r="7" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="17"/>
+      <c r="L5" s="17"/>
+      <c r="M5" s="17"/>
+      <c r="N5" s="17"/>
+      <c r="O5" s="17"/>
+      <c r="P5" s="17"/>
+      <c r="Q5" s="17"/>
+      <c r="R5" s="17"/>
+    </row>
+    <row r="6" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B6" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C6" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="17"/>
+      <c r="N6" s="17"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
+    </row>
+    <row r="7" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="B7" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="C7" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="D7" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="E7" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="5"/>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="5"/>
-    </row>
-    <row r="8" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9" t="s">
+      <c r="F7" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="G7" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="E8" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="G8" s="9" t="s">
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="17"/>
+      <c r="L7" s="17"/>
+      <c r="M7" s="17"/>
+      <c r="N7" s="17"/>
+      <c r="O7" s="17"/>
+      <c r="P7" s="17"/>
+      <c r="Q7" s="17"/>
+      <c r="R7" s="17"/>
+    </row>
+    <row r="8" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-      <c r="O8" s="5"/>
-      <c r="P8" s="5"/>
-      <c r="Q8" s="5"/>
-    </row>
-    <row r="9" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="D8" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="E8" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="G8" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="17"/>
+      <c r="L8" s="17"/>
+      <c r="M8" s="17"/>
+      <c r="N8" s="17"/>
+      <c r="O8" s="17"/>
+      <c r="P8" s="17"/>
+      <c r="Q8" s="17"/>
+      <c r="R8" s="17"/>
+    </row>
+    <row r="9" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="B9" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="E9" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F9" s="9" t="s">
+      <c r="C9" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="D9" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="5"/>
-      <c r="P9" s="5"/>
-      <c r="Q9" s="5"/>
-    </row>
-    <row r="10" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+      <c r="E9" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F9" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="G9" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="17"/>
+      <c r="M9" s="17"/>
+      <c r="N9" s="17"/>
+      <c r="O9" s="17"/>
+      <c r="P9" s="17"/>
+      <c r="Q9" s="17"/>
+      <c r="R9" s="17"/>
+    </row>
+    <row r="10" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="16" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="B10" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="E10" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F10" s="9" t="s">
+      <c r="C10" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="D10" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="5"/>
-      <c r="P10" s="5"/>
-      <c r="Q10" s="5"/>
-    </row>
-    <row r="11" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
+      <c r="E10" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="G10" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="17"/>
+      <c r="M10" s="17"/>
+      <c r="N10" s="17"/>
+      <c r="O10" s="17"/>
+      <c r="P10" s="17"/>
+      <c r="Q10" s="17"/>
+      <c r="R10" s="17"/>
+    </row>
+    <row r="11" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="B11" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="C11" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="D11" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="E11" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5"/>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="5"/>
-    </row>
-    <row r="12" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9" t="s">
+      <c r="F11" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="G11" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
+      <c r="L11" s="17"/>
+      <c r="M11" s="17"/>
+      <c r="N11" s="17"/>
+      <c r="O11" s="17"/>
+      <c r="P11" s="17"/>
+      <c r="Q11" s="17"/>
+      <c r="R11" s="17"/>
+    </row>
+    <row r="12" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="F12" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="G12" s="9" t="s">
+      <c r="D12" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="5"/>
-      <c r="P12" s="5"/>
-      <c r="Q12" s="5"/>
-    </row>
-    <row r="13" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
+      <c r="E12" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="F12" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="G12" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="17"/>
+      <c r="L12" s="17"/>
+      <c r="M12" s="17"/>
+      <c r="N12" s="17"/>
+      <c r="O12" s="17"/>
+      <c r="P12" s="17"/>
+      <c r="Q12" s="17"/>
+      <c r="R12" s="17"/>
+    </row>
+    <row r="13" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="B13" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="C13" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="F13" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="G13" s="9" t="s">
+      <c r="D13" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
-      <c r="P13" s="5"/>
-      <c r="Q13" s="5"/>
-    </row>
-    <row r="14" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+      <c r="E13" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="F13" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="G13" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="17"/>
+      <c r="M13" s="17"/>
+      <c r="N13" s="17"/>
+      <c r="O13" s="17"/>
+      <c r="P13" s="17"/>
+      <c r="Q13" s="17"/>
+      <c r="R13" s="17"/>
+    </row>
+    <row r="14" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="B14" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="E14" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F14" s="9" t="s">
+      <c r="C14" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="D14" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="5"/>
-      <c r="Q14" s="5"/>
-    </row>
-    <row r="15" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
+      <c r="E14" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" s="16" t="s">
         <v>138</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="G14" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17"/>
+      <c r="M14" s="17"/>
+      <c r="N14" s="17"/>
+      <c r="O14" s="17"/>
+      <c r="P14" s="17"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="17"/>
+    </row>
+    <row r="15" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="16" t="s">
         <v>140</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="B15" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="C15" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="D15" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="E15" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-      <c r="O15" s="5"/>
-      <c r="P15" s="5"/>
-      <c r="Q15" s="5"/>
-    </row>
-    <row r="16" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9" t="s">
+      <c r="F15" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="G15" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="E16" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="G16" s="9" t="s">
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="17"/>
+      <c r="M15" s="17"/>
+      <c r="N15" s="17"/>
+      <c r="O15" s="17"/>
+      <c r="P15" s="17"/>
+      <c r="Q15" s="17"/>
+      <c r="R15" s="17"/>
+    </row>
+    <row r="16" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="16"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-      <c r="N16" s="5"/>
-      <c r="O16" s="5"/>
-      <c r="P16" s="5"/>
-      <c r="Q16" s="5"/>
-    </row>
-    <row r="17" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
+      <c r="D16" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="E16" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>145</v>
+      </c>
+      <c r="G16" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="17"/>
+      <c r="K16" s="17"/>
+      <c r="L16" s="17"/>
+      <c r="M16" s="17"/>
+      <c r="N16" s="17"/>
+      <c r="O16" s="17"/>
+      <c r="P16" s="17"/>
+      <c r="Q16" s="17"/>
+      <c r="R16" s="17"/>
+    </row>
+    <row r="17" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="B17" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="C17" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="D17" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="E17" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-      <c r="O17" s="5"/>
-      <c r="P17" s="5"/>
-      <c r="Q17" s="5"/>
-    </row>
-    <row r="18" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9" t="s">
+      <c r="F17" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="G17" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="17"/>
+      <c r="M17" s="17"/>
+      <c r="N17" s="17"/>
+      <c r="O17" s="17"/>
+      <c r="P17" s="17"/>
+      <c r="Q17" s="17"/>
+      <c r="R17" s="17"/>
+    </row>
+    <row r="18" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="16"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="F18" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="G18" s="9" t="s">
+      <c r="D18" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-      <c r="N18" s="5"/>
-      <c r="O18" s="5"/>
-      <c r="P18" s="5"/>
-      <c r="Q18" s="5"/>
-    </row>
-    <row r="19" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
+      <c r="E18" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="F18" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="G18" s="16" t="s">
         <v>160</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="17"/>
+      <c r="L18" s="17"/>
+      <c r="M18" s="17"/>
+      <c r="N18" s="17"/>
+      <c r="O18" s="17"/>
+      <c r="P18" s="17"/>
+      <c r="Q18" s="17"/>
+      <c r="R18" s="17"/>
+    </row>
+    <row r="19" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="B19" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="E19" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F19" s="9" t="s">
+      <c r="C19" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="D19" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
-      <c r="P19" s="5"/>
-      <c r="Q19" s="5"/>
-    </row>
-    <row r="20" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
+      <c r="E19" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F19" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="G19" s="16" t="s">
         <v>166</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="17"/>
+      <c r="L19" s="17"/>
+      <c r="M19" s="17"/>
+      <c r="N19" s="17"/>
+      <c r="O19" s="17"/>
+      <c r="P19" s="17"/>
+      <c r="Q19" s="17"/>
+      <c r="R19" s="17"/>
+    </row>
+    <row r="20" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="B20" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="E20" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F20" s="9" t="s">
+      <c r="C20" s="16" t="s">
         <v>169</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="D20" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5"/>
-      <c r="P20" s="5"/>
-      <c r="Q20" s="5"/>
-    </row>
-    <row r="21" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="9" t="s">
+      <c r="E20" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F20" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="G20" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="17"/>
+      <c r="M20" s="17"/>
+      <c r="N20" s="17"/>
+      <c r="O20" s="17"/>
+      <c r="P20" s="17"/>
+      <c r="Q20" s="17"/>
+      <c r="R20" s="17"/>
+    </row>
+    <row r="21" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="B21" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="E21" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F21" s="9" t="s">
+      <c r="C21" s="16" t="s">
         <v>175</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="D21" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5"/>
-      <c r="P21" s="5"/>
-      <c r="Q21" s="5"/>
-    </row>
-    <row r="22" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="9" t="s">
+      <c r="E21" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F21" s="16" t="s">
         <v>177</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="G21" s="16" t="s">
         <v>178</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="17"/>
+      <c r="M21" s="17"/>
+      <c r="N21" s="17"/>
+      <c r="O21" s="17"/>
+      <c r="P21" s="17"/>
+      <c r="Q21" s="17"/>
+      <c r="R21" s="17"/>
+    </row>
+    <row r="22" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="16" t="s">
         <v>179</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="B22" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="C22" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="D22" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="G22" s="9" t="s">
+      <c r="E22" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
-      <c r="N22" s="5"/>
-      <c r="O22" s="5"/>
-      <c r="P22" s="5"/>
-      <c r="Q22" s="5"/>
-    </row>
-    <row r="23" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="9"/>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9" t="s">
+      <c r="F22" s="16" t="s">
         <v>184</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="G22" s="16" t="s">
         <v>185</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="17"/>
+      <c r="K22" s="17"/>
+      <c r="L22" s="17"/>
+      <c r="M22" s="17"/>
+      <c r="N22" s="17"/>
+      <c r="O22" s="17"/>
+      <c r="P22" s="17"/>
+      <c r="Q22" s="17"/>
+      <c r="R22" s="17"/>
+    </row>
+    <row r="23" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="16"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="16" t="s">
         <v>186</v>
       </c>
-      <c r="F23" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="G23" s="9" t="s">
+      <c r="D23" s="16" t="s">
         <v>187</v>
       </c>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="5"/>
-      <c r="O23" s="5"/>
-      <c r="P23" s="5"/>
-      <c r="Q23" s="5"/>
-    </row>
-    <row r="24" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
+      <c r="E23" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="F23" s="16" t="s">
+        <v>184</v>
+      </c>
+      <c r="G23" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="17"/>
+      <c r="M23" s="17"/>
+      <c r="N23" s="17"/>
+      <c r="O23" s="17"/>
+      <c r="P23" s="17"/>
+      <c r="Q23" s="17"/>
+      <c r="R23" s="17"/>
+    </row>
+    <row r="24" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="16" t="s">
         <v>190</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="B24" s="16" t="s">
         <v>191</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="C24" s="16" t="s">
         <v>192</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="D24" s="16" t="s">
         <v>193</v>
       </c>
-      <c r="G24" s="9" t="s">
+      <c r="E24" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
-      <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
-      <c r="N24" s="5"/>
-      <c r="O24" s="5"/>
-      <c r="P24" s="5"/>
-      <c r="Q24" s="5"/>
-    </row>
-    <row r="25" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="9"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9" t="s">
+      <c r="F24" s="16" t="s">
         <v>195</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="G24" s="16" t="s">
         <v>196</v>
       </c>
-      <c r="E25" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="G25" s="9" t="s">
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="17"/>
+      <c r="M24" s="17"/>
+      <c r="N24" s="17"/>
+      <c r="O24" s="17"/>
+      <c r="P24" s="17"/>
+      <c r="Q24" s="17"/>
+      <c r="R24" s="17"/>
+    </row>
+    <row r="25" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="16"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
-      <c r="L25" s="5"/>
-      <c r="M25" s="5"/>
-      <c r="N25" s="5"/>
-      <c r="O25" s="5"/>
-      <c r="P25" s="5"/>
-      <c r="Q25" s="5"/>
-    </row>
-    <row r="26" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="9" t="s">
+      <c r="D25" s="16" t="s">
         <v>198</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="E25" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F25" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="G25" s="16" t="s">
         <v>199</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="17"/>
+      <c r="M25" s="17"/>
+      <c r="N25" s="17"/>
+      <c r="O25" s="17"/>
+      <c r="P25" s="17"/>
+      <c r="Q25" s="17"/>
+      <c r="R25" s="17"/>
+    </row>
+    <row r="26" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="16" t="s">
         <v>200</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="B26" s="16" t="s">
         <v>201</v>
       </c>
-      <c r="E26" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F26" s="9" t="s">
+      <c r="C26" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="G26" s="9" t="s">
+      <c r="D26" s="16" t="s">
         <v>203</v>
       </c>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
-      <c r="L26" s="5"/>
-      <c r="M26" s="5"/>
-      <c r="N26" s="5"/>
-      <c r="O26" s="5"/>
-      <c r="P26" s="5"/>
-      <c r="Q26" s="5"/>
-    </row>
-    <row r="27" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="9" t="s">
+      <c r="E26" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F26" s="16" t="s">
         <v>204</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="G26" s="16" t="s">
         <v>205</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="17"/>
+      <c r="K26" s="17"/>
+      <c r="L26" s="17"/>
+      <c r="M26" s="17"/>
+      <c r="N26" s="17"/>
+      <c r="O26" s="17"/>
+      <c r="P26" s="17"/>
+      <c r="Q26" s="17"/>
+      <c r="R26" s="17"/>
+    </row>
+    <row r="27" spans="1:18" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="B27" s="16" t="s">
         <v>207</v>
       </c>
-      <c r="E27" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F27" s="9" t="s">
+      <c r="C27" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="D27" s="16" t="s">
         <v>209</v>
       </c>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
-      <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
-      <c r="N27" s="5"/>
-      <c r="O27" s="5"/>
-      <c r="P27" s="5"/>
-      <c r="Q27" s="5"/>
+      <c r="E27" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F27" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="G27" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="17"/>
+      <c r="L27" s="17"/>
+      <c r="M27" s="17"/>
+      <c r="N27" s="17"/>
+      <c r="O27" s="17"/>
+      <c r="P27" s="17"/>
+      <c r="Q27" s="17"/>
+      <c r="R27" s="17"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q1"/>
+  <autoFilter ref="A1:R27"/>
   <mergeCells count="48">
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="B7:B8"/>
-    <mergeCell ref="L7:L8"/>
     <mergeCell ref="M7:M8"/>
     <mergeCell ref="N7:N8"/>
     <mergeCell ref="O7:O8"/>
     <mergeCell ref="P7:P8"/>
     <mergeCell ref="Q7:Q8"/>
+    <mergeCell ref="R7:R8"/>
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="B11:B12"/>
-    <mergeCell ref="L11:L12"/>
     <mergeCell ref="M11:M12"/>
     <mergeCell ref="N11:N12"/>
     <mergeCell ref="O11:O12"/>
     <mergeCell ref="P11:P12"/>
     <mergeCell ref="Q11:Q12"/>
+    <mergeCell ref="R11:R12"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="B15:B16"/>
-    <mergeCell ref="L15:L16"/>
     <mergeCell ref="M15:M16"/>
     <mergeCell ref="N15:N16"/>
     <mergeCell ref="O15:O16"/>
     <mergeCell ref="P15:P16"/>
     <mergeCell ref="Q15:Q16"/>
+    <mergeCell ref="R15:R16"/>
     <mergeCell ref="A17:A18"/>
     <mergeCell ref="B17:B18"/>
-    <mergeCell ref="L17:L18"/>
     <mergeCell ref="M17:M18"/>
     <mergeCell ref="N17:N18"/>
     <mergeCell ref="O17:O18"/>
     <mergeCell ref="P17:P18"/>
     <mergeCell ref="Q17:Q18"/>
+    <mergeCell ref="R17:R18"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="B22:B23"/>
-    <mergeCell ref="L22:L23"/>
     <mergeCell ref="M22:M23"/>
     <mergeCell ref="N22:N23"/>
     <mergeCell ref="O22:O23"/>
     <mergeCell ref="P22:P23"/>
     <mergeCell ref="Q22:Q23"/>
+    <mergeCell ref="R22:R23"/>
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="B24:B25"/>
-    <mergeCell ref="L24:L25"/>
     <mergeCell ref="M24:M25"/>
     <mergeCell ref="N24:N25"/>
     <mergeCell ref="O24:O25"/>
     <mergeCell ref="P24:P25"/>
     <mergeCell ref="Q24:Q25"/>
+    <mergeCell ref="R24:R25"/>
   </mergeCells>
   <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" sqref="H10:H27">
@@ -2330,16 +2439,16 @@
     <dataValidation type="list" allowBlank="1" sqref="H7:H27">
       <formula1>"verifisert,delvis,sekundær,ikke funnet,feil"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="J10:J27">
+    <dataValidation type="list" allowBlank="1" sqref="K10:K27">
       <formula1>"ja,nei,preprint"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="J2:J27">
+    <dataValidation type="list" allowBlank="1" sqref="K2:K27">
       <formula1>"ja,nei,preprint"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L10:P27">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M10:Q27">
       <formula1>"0,1,2,3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L2:P27">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M2:Q27">
       <formula1>"0,1,2,3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>